<commit_message>
Updated to be compatible with new food_as_industry scenario workbook
</commit_message>
<xml_diff>
--- a/data/scenarios/no_cows.xlsx
+++ b/data/scenarios/no_cows.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="28">
   <si>
     <t>f_food</t>
   </si>
@@ -95,13 +95,22 @@
   </si>
   <si>
     <t>semi-natural grasslands</t>
+  </si>
+  <si>
+    <t>export_demand</t>
+  </si>
+  <si>
+    <t>Milk powder</t>
+  </si>
+  <si>
+    <t>Exports</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,8 +133,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -135,6 +150,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -151,13 +172,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,7 +551,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" bestFit="1" customWidth="1"/>
@@ -740,6 +764,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>